<commit_message>
Align store policies and refresh all handoff documents
</commit_message>
<xml_diff>
--- a/outputs/01a0f4e1-9633-7ef3-9ea3-45372f0331d8/말마프렌즈_온라인스토어_최종_IA_기능명세_기본견적.xlsx
+++ b/outputs/01a0f4e1-9633-7ef3-9ea3-45372f0331d8/말마프렌즈_온라인스토어_최종_IA_기능명세_기본견적.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="Rd98f0889c5aa4d23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IA" sheetId="2" r:id="R1ae9302719a74e30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기능명세" sheetId="3" r:id="R07cc87ccfa50426f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기본견적" sheetId="4" r:id="R1173729199f14d3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객사 협의" sheetId="5" r:id="R98acb47b37f04253"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="요약" sheetId="1" r:id="R6d63d7a6c61c4224"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="IA" sheetId="2" r:id="R0678fccb85274cd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기능명세" sheetId="3" r:id="R6edbb711fbd3431f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="기본견적" sheetId="4" r:id="Reeca75370cbb4ca4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="고객사 협의" sheetId="5" r:id="R325c13928a784fd4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -445,7 +445,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>IA · 기능명세 · 기본 견적 | 확정 정책 2026-10-01</x:v>
+        <x:v>IA와 기능명세 및 기본 견적 · 정책 개정 2026-10-07</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -588,7 +588,7 @@
         <x:v>환불·반려·예외 환불</x:v>
       </x:c>
       <x:c r="D13" s="16" t="str">
-        <x:v>상품 부분 반품 없음</x:v>
+        <x:v>주문 전체 반품</x:v>
       </x:c>
       <x:c r="E13" s="16" t="str">
         <x:v>환불월 차감</x:v>
@@ -608,13 +608,13 @@
         <x:v>주문별 송장 등록·수정</x:v>
       </x:c>
       <x:c r="D14" s="16" t="str">
-        <x:v>삭제·수정 이력 없음</x:v>
+        <x:v>등록 정보는 최신값으로 수정</x:v>
       </x:c>
       <x:c r="E14" s="16" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F14" s="16" t="str">
-        <x:v>일괄 배송 제외</x:v>
+        <x:v>주문별 처리</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
@@ -628,7 +628,7 @@
         <x:v>수동 상태 관리</x:v>
       </x:c>
       <x:c r="D15" s="16" t="str">
-        <x:v>결제 전 선점 없음</x:v>
+        <x:v>승인 순서 재고 차감</x:v>
       </x:c>
       <x:c r="E15" s="16" t="str">
         <x:v>—</x:v>
@@ -671,21 +671,21 @@
         <x:v>통합 관리자 기본</x:v>
       </x:c>
       <x:c r="E17" s="16" t="str">
-        <x:v>개인정보 미노출</x:v>
+        <x:v>주문 정보 중심 원장</x:v>
       </x:c>
       <x:c r="F17" s="16" t="str">
         <x:v>포함</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="15" hidden="0" customHeight="1">
+    <x:row r="18" ht="32" hidden="0" customHeight="1">
       <x:c r="A18" s="19" t="str">
         <x:v>목록</x:v>
       </x:c>
       <x:c r="B18" s="16" t="str">
-        <x:v>—</x:v>
+        <x:v>상품 24개 · 주문 10건 / 페이지</x:v>
       </x:c>
       <x:c r="C18" s="16" t="str">
-        <x:v>20건/페이지</x:v>
+        <x:v>관리자 20건 / 페이지</x:v>
       </x:c>
       <x:c r="D18" s="16" t="str">
         <x:v>필터 변경 시 1페이지</x:v>
@@ -699,22 +699,22 @@
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="19" t="str">
-        <x:v>알림</x:v>
+        <x:v>고객 안내</x:v>
       </x:c>
       <x:c r="B19" s="16" t="str">
         <x:v>화면 상태 확인</x:v>
       </x:c>
       <x:c r="C19" s="16" t="str">
-        <x:v>기존 CS 처리</x:v>
+        <x:v>기존 고객센터 후속 처리</x:v>
       </x:c>
       <x:c r="D19" s="16" t="str">
-        <x:v>자동 알림 없음</x:v>
+        <x:v>처리 결과 화면 표시</x:v>
       </x:c>
       <x:c r="E19" s="16" t="str">
         <x:v>—</x:v>
       </x:c>
       <x:c r="F19" s="16" t="str">
-        <x:v>제외</x:v>
+        <x:v>기본</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1114,7 +1114,7 @@
         <x:v>확정 동작</x:v>
       </x:c>
       <x:c r="E4" s="12" t="str">
-        <x:v>예외/검증</x:v>
+        <x:v>검증과 처리</x:v>
       </x:c>
       <x:c r="F4" s="12" t="str">
         <x:v>상태</x:v>
@@ -1122,7 +1122,7 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="16" t="str">
-        <x:v>FN-001</x:v>
+        <x:v>FN-025</x:v>
       </x:c>
       <x:c r="B5" s="16" t="str">
         <x:v>상품</x:v>
@@ -1134,7 +1134,7 @@
         <x:v>관리자 수동 순서, 신규는 마지막, 품절도 위치 유지</x:v>
       </x:c>
       <x:c r="E5" s="16" t="str">
-        <x:v>편집·재입고로 자동 이동하지 않음</x:v>
+        <x:v>편집·재입고 후 기존 순서 유지</x:v>
       </x:c>
       <x:c r="F5" s="22" t="str">
         <x:v>확정</x:v>
@@ -1142,7 +1142,7 @@
     </x:row>
     <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="16" t="str">
-        <x:v>FN-002</x:v>
+        <x:v>FN-022</x:v>
       </x:c>
       <x:c r="B6" s="16" t="str">
         <x:v>상품</x:v>
@@ -1162,7 +1162,7 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0" customHeight="1">
       <x:c r="A7" s="16" t="str">
-        <x:v>FN-003</x:v>
+        <x:v>FN-023</x:v>
       </x:c>
       <x:c r="B7" s="16" t="str">
         <x:v>상품</x:v>
@@ -1174,7 +1174,7 @@
         <x:v>서식·링크·이미지·영상 URL·미리보기</x:v>
       </x:c>
       <x:c r="E7" s="16" t="str">
-        <x:v>영상 파일 직접 업로드 제외</x:v>
+        <x:v>상세 콘텐츠 미리보기와 HTML 정제</x:v>
       </x:c>
       <x:c r="F7" s="22" t="str">
         <x:v>확정</x:v>
@@ -1182,7 +1182,7 @@
     </x:row>
     <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="16" t="str">
-        <x:v>FN-004</x:v>
+        <x:v>FN-006</x:v>
       </x:c>
       <x:c r="B8" s="16" t="str">
         <x:v>장바구니</x:v>
@@ -1202,7 +1202,7 @@
     </x:row>
     <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="16" t="str">
-        <x:v>FN-005</x:v>
+        <x:v>FN-009</x:v>
       </x:c>
       <x:c r="B9" s="16" t="str">
         <x:v>결제</x:v>
@@ -1211,7 +1211,7 @@
         <x:v>가격·재고 재검증</x:v>
       </x:c>
       <x:c r="D9" s="16" t="str">
-        <x:v>승인 순서 원자적 차감, 선점 없음</x:v>
+        <x:v>승인 순서대로 재고 원자적 차감</x:v>
       </x:c>
       <x:c r="E9" s="16" t="str">
         <x:v>동시 소진 후속 승인 자동 전액 취소</x:v>
@@ -1222,7 +1222,7 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="16" t="str">
-        <x:v>FN-006</x:v>
+        <x:v>FN-008</x:v>
       </x:c>
       <x:c r="B10" s="16" t="str">
         <x:v>동의</x:v>
@@ -1242,7 +1242,7 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0" customHeight="1">
       <x:c r="A11" s="16" t="str">
-        <x:v>FN-007</x:v>
+        <x:v>FN-013 / FN-018</x:v>
       </x:c>
       <x:c r="B11" s="16" t="str">
         <x:v>취소</x:v>
@@ -1254,7 +1254,7 @@
         <x:v>고객 24시간 기본+발송 전, 관리자는 발송 전 언제든</x:v>
       </x:c>
       <x:c r="E11" s="16" t="str">
-        <x:v>전액 환불·재고 복원, 판매 자동 재개 없음</x:v>
+        <x:v>취소 재고 복원 후 판매 상태 유지</x:v>
       </x:c>
       <x:c r="F11" s="22" t="str">
         <x:v>확정</x:v>
@@ -1262,7 +1262,7 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0" customHeight="1">
       <x:c r="A12" s="16" t="str">
-        <x:v>FN-008</x:v>
+        <x:v>FN-019 / FN-020</x:v>
       </x:c>
       <x:c r="B12" s="16" t="str">
         <x:v>배송</x:v>
@@ -1274,7 +1274,7 @@
         <x:v>주문별 등록·수정, 기본 택배사+건별 변경</x:v>
       </x:c>
       <x:c r="E12" s="16" t="str">
-        <x:v>중복 허용, 삭제·수정 이력 없음</x:v>
+        <x:v>공백·하이픈 제거, 영문·숫자 허용</x:v>
       </x:c>
       <x:c r="F12" s="22" t="str">
         <x:v>확정</x:v>
@@ -1282,7 +1282,7 @@
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
       <x:c r="A13" s="16" t="str">
-        <x:v>FN-009</x:v>
+        <x:v>FN-014</x:v>
       </x:c>
       <x:c r="B13" s="16" t="str">
         <x:v>반품</x:v>
@@ -1294,7 +1294,7 @@
         <x:v>최초 송장 등록부터 14일 기본, 고객 직접 반송</x:v>
       </x:c>
       <x:c r="E13" s="16" t="str">
-        <x:v>상품·수량 일부 반품 없음</x:v>
+        <x:v>기한 내 주문 전체 반품</x:v>
       </x:c>
       <x:c r="F13" s="22" t="str">
         <x:v>확정</x:v>
@@ -1302,7 +1302,7 @@
     </x:row>
     <x:row r="14" ht="15" hidden="0" customHeight="1">
       <x:c r="A14" s="16" t="str">
-        <x:v>FN-010</x:v>
+        <x:v>FN-017</x:v>
       </x:c>
       <x:c r="B14" s="16" t="str">
         <x:v>환불</x:v>
@@ -1314,7 +1314,7 @@
         <x:v>전액 또는 배송비 차감, 안내 자동 생성+추가 문구</x:v>
       </x:c>
       <x:c r="E14" s="16" t="str">
-        <x:v>재고 미복원, 완료 후 변경 불가</x:v>
+        <x:v>현재 재고와 확정 결과 유지</x:v>
       </x:c>
       <x:c r="F14" s="22" t="str">
         <x:v>확정</x:v>
@@ -1322,7 +1322,7 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="16" t="str">
-        <x:v>FN-011</x:v>
+        <x:v>FN-017</x:v>
       </x:c>
       <x:c r="B15" s="16" t="str">
         <x:v>반품</x:v>
@@ -1334,7 +1334,7 @@
         <x:v>필수 사유 고객 표시, 재신청 차단</x:v>
       </x:c>
       <x:c r="E15" s="16" t="str">
-        <x:v>재발송 송장 없음, 이후 CS</x:v>
+        <x:v>고객센터 후속 처리</x:v>
       </x:c>
       <x:c r="F15" s="22" t="str">
         <x:v>확정</x:v>
@@ -1342,7 +1342,7 @@
     </x:row>
     <x:row r="16" ht="15" hidden="0" customHeight="1">
       <x:c r="A16" s="16" t="str">
-        <x:v>FN-012</x:v>
+        <x:v>FN-018</x:v>
       </x:c>
       <x:c r="B16" s="16" t="str">
         <x:v>환불</x:v>
@@ -1354,7 +1354,7 @@
         <x:v>발송 후 반품 없이 전액/배송비 차감, 내부 사유 필수</x:v>
       </x:c>
       <x:c r="E16" s="16" t="str">
-        <x:v>재고 미복원, 완료 후 변경 불가</x:v>
+        <x:v>현재 재고와 확정 결과 유지</x:v>
       </x:c>
       <x:c r="F16" s="22" t="str">
         <x:v>확정</x:v>
@@ -1362,7 +1362,7 @@
     </x:row>
     <x:row r="17" ht="15" hidden="0" customHeight="1">
       <x:c r="A17" s="16" t="str">
-        <x:v>FN-013</x:v>
+        <x:v>FN-026</x:v>
       </x:c>
       <x:c r="B17" s="16" t="str">
         <x:v>설정</x:v>
@@ -1380,9 +1380,9 @@
         <x:v>확정</x:v>
       </x:c>
     </x:row>
-    <x:row r="18" ht="15" hidden="0" customHeight="1">
+    <x:row r="18" ht="34" hidden="0" customHeight="1">
       <x:c r="A18" s="16" t="str">
-        <x:v>FN-014</x:v>
+        <x:v>FN-015 / FN-016</x:v>
       </x:c>
       <x:c r="B18" s="16" t="str">
         <x:v>목록</x:v>
@@ -1391,10 +1391,10 @@
         <x:v>검색·페이지·다운로드</x:v>
       </x:c>
       <x:c r="D18" s="16" t="str">
-        <x:v>주문번호·상품명 검색, 20건/페이지</x:v>
+        <x:v>상품 24개 · 본인 주문 10건 · 관리자 20건 / 페이지</x:v>
       </x:c>
       <x:c r="E18" s="16" t="str">
-        <x:v>필터 변경 1페이지, 다운로드 전체 결과</x:v>
+        <x:v>조건 변경 시 1페이지, 전체 결과 다운로드</x:v>
       </x:c>
       <x:c r="F18" s="22" t="str">
         <x:v>확정</x:v>
@@ -1402,7 +1402,7 @@
     </x:row>
     <x:row r="19" ht="15" hidden="0" customHeight="1">
       <x:c r="A19" s="16" t="str">
-        <x:v>FN-015</x:v>
+        <x:v>FN-027</x:v>
       </x:c>
       <x:c r="B19" s="16" t="str">
         <x:v>정산</x:v>
@@ -1411,7 +1411,7 @@
         <x:v>월 정산</x:v>
       </x:c>
       <x:c r="D19" s="16" t="str">
-        <x:v>승인월, 익월 8일, PG 2%, 환불 익월 차감</x:v>
+        <x:v>승인월, 익월 8일, PG 2%, 환불 완료월 조정</x:v>
       </x:c>
       <x:c r="E19" s="16" t="str">
         <x:v>휴일 다음 영업일, 음수 차감 이월</x:v>
@@ -1422,7 +1422,7 @@
     </x:row>
     <x:row r="20" ht="15" hidden="0" customHeight="1">
       <x:c r="A20" s="16" t="str">
-        <x:v>FN-016</x:v>
+        <x:v>FN-028</x:v>
       </x:c>
       <x:c r="B20" s="16" t="str">
         <x:v>권한</x:v>
@@ -1431,7 +1431,7 @@
         <x:v>커머스 관리자 권한</x:v>
       </x:c>
       <x:c r="D20" s="16" t="str">
-        <x:v>계정별 boolean, 통합 관리자 기본 true</x:v>
+        <x:v>계정별 권한 부여, 통합 관리자 기본 부여</x:v>
       </x:c>
       <x:c r="E20" s="16" t="str">
         <x:v>기존 지역·부서 권한과 분리</x:v>
@@ -1469,7 +1469,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="6" t="str">
-        <x:v>수정 견적서 기준 · 커머스 정산 포함</x:v>
+        <x:v>기본 견적과 포함 기능 · 정책 개정 2026-10-07</x:v>
       </x:c>
       <x:c r="B2" s="6"/>
       <x:c r="C2" s="6"/>
@@ -1630,7 +1630,7 @@
         <x:v>포함</x:v>
       </x:c>
       <x:c r="C17" s="12" t="str">
-        <x:v>제외</x:v>
+        <x:v>처리 기준</x:v>
       </x:c>
       <x:c r="D17" s="12" t="str">
         <x:v>산정 메모</x:v>
@@ -1644,7 +1644,7 @@
         <x:v>목록·상세·장바구니·결제·주문조회·전체 취소·전체 반품</x:v>
       </x:c>
       <x:c r="C18" s="16" t="str">
-        <x:v>비회원·해외·쿠폰·옵션</x:v>
+        <x:v>회원 로그인 후 구매</x:v>
       </x:c>
       <x:c r="D18" s="16" t="str">
         <x:v>기존 회원·PG 연동</x:v>
@@ -1658,7 +1658,7 @@
         <x:v>상품·배너·설정·주문·배송·반품·예외 환불</x:v>
       </x:c>
       <x:c r="C19" s="16" t="str">
-        <x:v>일괄 배송·자동 알림</x:v>
+        <x:v>주문별 배송·환불·반려</x:v>
       </x:c>
       <x:c r="D19" s="16" t="str">
         <x:v>계정별 권한 포함</x:v>
@@ -1672,10 +1672,10 @@
         <x:v>월 원장·2% 수수료·환불 조정·이월·XLSX</x:v>
       </x:c>
       <x:c r="C20" s="16" t="str">
-        <x:v>송금·지급완료 처리</x:v>
+        <x:v>익월 지급 예정·차감 이월</x:v>
       </x:c>
       <x:c r="D20" s="16" t="str">
-        <x:v>개인정보 제외</x:v>
+        <x:v>주문 정보 중심 원장</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="24" hidden="0" customHeight="1">
@@ -1686,7 +1686,7 @@
         <x:v>서식·링크·이미지·영상 URL·미리보기</x:v>
       </x:c>
       <x:c r="C21" s="16" t="str">
-        <x:v>영상 파일 업로드</x:v>
+        <x:v>외부 영상 주소 삽입</x:v>
       </x:c>
       <x:c r="D21" s="16" t="str">
         <x:v>기본 범위</x:v>
@@ -1700,10 +1700,10 @@
         <x:v>승인 순 차감·취소 복원·수동 조정</x:v>
       </x:c>
       <x:c r="C22" s="16" t="str">
-        <x:v>결제 전 선점</x:v>
+        <x:v>승인 완료 순서로 차감</x:v>
       </x:c>
       <x:c r="D22" s="16" t="str">
-        <x:v>반품 재고 자동복원 제외</x:v>
+        <x:v>반품·예외 환불은 현재 재고 유지</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="15" hidden="0" customHeight="1">
@@ -1714,7 +1714,7 @@
         <x:v>주문별 송장 등록·수정</x:v>
       </x:c>
       <x:c r="C23" s="16" t="str">
-        <x:v>엑셀 업로드·일괄 처리</x:v>
+        <x:v>영문·숫자 송장 등록</x:v>
       </x:c>
       <x:c r="D23" s="16" t="str">
         <x:v>발송 완료까지만</x:v>
@@ -1802,7 +1802,7 @@
         <x:v>개인정보 보존·삭제 기간</x:v>
       </x:c>
       <x:c r="C5" s="16" t="str">
-        <x:v>정산 화면·XLSX에는 개인정보 미포함</x:v>
+        <x:v>정산 원장은 주문·상품·금액·상태로 구성</x:v>
       </x:c>
       <x:c r="D5" s="16" t="str">
         <x:v>주문·배송·내려받기 자료의 보존기간, 파기 시점과 방식</x:v>

</xml_diff>